<commit_message>
Corrected the type in the example metadata file/worksheet
</commit_message>
<xml_diff>
--- a/doc/_static/example-files/YES-INVITATION-1-0-client-completed-treatment.xlsx
+++ b/doc/_static/example-files/YES-INVITATION-1-0-client-completed-treatment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jennib/Work/git/PMHC/spec-yes-invitation/doc/_static/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jennib/Work/git/PMHC/spec-yes-invitation/doc/_static/example-files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C47B194-F018-7B46-86C9-B9A6757BF898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621F4C43-DE90-DF4C-A9AF-7D0E8FB183F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="760" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="16100" windowHeight="9660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -32,9 +32,6 @@
     <t>type</t>
   </si>
   <si>
-    <t>omsss-invitations</t>
-  </si>
-  <si>
     <t>version</t>
   </si>
   <si>
@@ -147,6 +144,9 @@
   </si>
   <si>
     <t>EP000034</t>
+  </si>
+  <si>
+    <t>YES-INVITATION</t>
   </si>
 </sst>
 </file>
@@ -508,12 +508,12 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -528,218 +528,223 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="12.5" customWidth="1"/>
+    <col min="4" max="4" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="49.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>11</v>
-      </c>
-      <c r="H1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
       </c>
       <c r="D2" s="1">
         <v>44181</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
       </c>
       <c r="D3" s="1">
         <v>43978</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
         <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
       </c>
       <c r="D4" s="1">
         <v>43968</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
         <v>23</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
       </c>
       <c r="D5" s="1">
         <v>43552</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
         <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
       </c>
       <c r="D6" s="1">
         <v>42826</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
         <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
       </c>
       <c r="D7" s="1">
         <v>42826</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>31</v>
-      </c>
-      <c r="C8" t="s">
-        <v>32</v>
       </c>
       <c r="D8" s="1">
         <v>42748</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
       </c>
       <c r="D9" s="1">
         <v>42712</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
         <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
       </c>
       <c r="D10" s="1">
         <v>42699</v>
       </c>
       <c r="E10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
         <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
       </c>
       <c r="D11" s="1">
         <v>42693</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
         <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
       </c>
       <c r="D12" s="1">
         <v>42689</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>